<commit_message>
Updated the query files to fetch data from memgraph db
</commit_message>
<xml_diff>
--- a/InputFiles/CDS/TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture.xlsx
+++ b/InputFiles/CDS/TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture.xlsx
@@ -1,45 +1,49 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kallakuriv2\Automation\sowjany0601\Commons_Automation\InputFiles\CDS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sohilz2/Automation/Commons_Automation/InputFiles/CDS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{818106A2-3DFE-434E-AEB8-4DD53DAFBA4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A79389-6B4C-7648-A6AB-51E24AEBF752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8362173B-D28C-47E7-8626-98E16101E601}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
+    <t>TabName</t>
+  </si>
+  <si>
+    <t>TabQuery</t>
+  </si>
+  <si>
+    <t>StatQuery</t>
+  </si>
+  <si>
+    <t>TsvExcel</t>
+  </si>
+  <si>
     <t>WebExcel</t>
   </si>
   <si>
-    <t>StatQuery</t>
-  </si>
-  <si>
-    <t>TabName</t>
+    <t>ParticipantsTab</t>
+  </si>
+  <si>
+    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_TSVData.xlsx</t>
+  </si>
+  <si>
+    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_WebData.xlsx</t>
   </si>
   <si>
     <t>SamplesTab</t>
@@ -48,223 +52,85 @@
     <t>FilesTab</t>
   </si>
   <si>
-    <t>ParticipantsTab</t>
-  </si>
-  <si>
-    <t>TabQuery</t>
-  </si>
-  <si>
-    <t>TsvExcel</t>
-  </si>
-  <si>
-    <t>WITH Filtered_Files AS (
-    SELECT DISTINCT f.file_id
-    FROM df_file f
-    JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_study s ON sp."study.phs_accession" = s.phs_accession
-    JOIN df_program p ON p.program_acronym = s."program.program_acronym"
-    JOIN df_diagnosis d ON d."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_genomic_info gi ON gi."file.file_id" = f.file_id
-    WHERE 
-        s.phs_accession = 'phs002599'
-        AND smp.sample_tumor_status = 'Not specified in data'
-        AND smp.sample_type = 'RNA'
-        AND gi.library_strategy = 'Targeted-Capture'),
-Matched_Participants AS (
-    SELECT DISTINCT sp.*
-    FROM Filtered_Files ff
-    JOIN df_file f ON f.file_id = ff.file_id
-    JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id),
-Matched_Samples AS (
-    SELECT DISTINCT smp.*
-    FROM Matched_Participants sp
-    JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-    WHERE 
-        smp.sample_tumor_status = 'Not specified in data'
-        AND smp.sample_type = 'RNA')
-SELECT 
-    COUNT(DISTINCT s.study_name) AS "Studies",
-    COUNT(DISTINCT sp.participant_id) AS "Participants",
-    COUNT(DISTINCT smp.sample_id) AS "Samples",
-    COUNT(DISTINCT f.file_id) AS "Files"
-FROM Filtered_Files ff
-JOIN df_file f ON f.file_id = ff.file_id
-JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id
-JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-    AND smp.sample_tumor_status = 'Not specified in data'
-    AND smp.sample_type = 'RNA'
-JOIN df_study s ON sp."study.phs_accession" = s.phs_accession
-JOIN df_program p ON p.program_acronym = s."program.program_acronym"
-JOIN df_diagnosis d ON d."participant.study_participant_id" = sp.study_participant_id
-JOIN df_genomic_info gi ON gi."file.file_id" = f.file_id;</t>
-  </si>
-  <si>
-    <t>WITH Filtered_Participants AS (
-    SELECT DISTINCT
-        sp.participant_id,
-        sp.study_participant_id,
-        sp.gender,
-        s.study_name,
-        s.phs_accession
-    FROM df_file f
-    JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_study s ON sp."study.phs_accession" = s.phs_accession
-    JOIN df_program p ON p.program_acronym = s."program.program_acronym"
-    JOIN df_diagnosis d ON d."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_genomic_info gi ON gi."file.file_id" = f.file_id
-    WHERE 
-         s.phs_accession = 'phs002599' 
-AND smp.sample_tumor_status = 'Not specified in data'
-AND smp.sample_type = 'RNA'
-AND gi.library_strategy = 'Targeted-Capture'
-),
-Participant_Samples AS (
-    SELECT DISTINCT
-        fp.participant_id,
-        fp.study_name,
-        fp.phs_accession,
-        fp.gender,
-        smp.sample_id
-    FROM Filtered_Participants fp
-    JOIN df_sample smp ON smp."participant.study_participant_id" = fp.study_participant_id
-),
-Numbered_Samples AS (
-    SELECT
-        participant_id,
-        study_name,
-        phs_accession,
-        gender,
-        sample_id,
-        ROW_NUMBER() OVER (PARTITION BY participant_id ORDER BY sample_id) AS rn
-    FROM Participant_Samples
-),
-Sample_Groups AS (
-    SELECT
-        participant_id,
-        study_name,
-        phs_accession,
-        gender,
-        COUNT(*) AS total_samples,
-        GROUP_CONCAT(sample_id, ', ') FILTER (WHERE rn &lt;= 5) AS sample_list
-    FROM Numbered_Samples
-    GROUP BY participant_id, study_name, phs_accession, gender
-)
-SELECT
-    participant_id AS "Participant ID",
-    study_name AS "Study Name",
-    phs_accession AS Accession,
-    gender AS gender,
-    CASE 
-        WHEN total_samples &gt; 5 THEN sample_list || ', ...'
-        ELSE sample_list
-    END AS Samples
-FROM Sample_Groups
-LIMIT 100;</t>
-  </si>
-  <si>
-    <t>WITH Filtered_Files AS (
-    SELECT DISTINCT f.file_id
-    FROM df_file f
-    JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-    JOIN df_study s ON sp."study.phs_accession" = s.phs_accession
-    JOIN df_genomic_info gi ON gi."file.file_id" = f.file_id
-    WHERE 
-        s.phs_accession = 'phs002599' 
-        AND smp.sample_tumor_status = 'Not specified in data'
-        AND smp.sample_type = 'RNA'
-        AND gi.library_strategy = 'Targeted-Capture'
-),
-Sample_List AS (
-    SELECT 
-        smp.sample_id,
-        smp."participant.study_participant_id",
-        ROW_NUMBER() OVER (
-            PARTITION BY smp."participant.study_participant_id"
-            ORDER BY smp.sample_id
-        ) AS rn
-    FROM df_sample smp
-)
-SELECT
-    f.file_name AS "File Name",
-    s.study_name AS "Study Name",
-    s.phs_accession AS "Accession",
-    sp.participant_id AS "Participant ID",
-    COALESCE((
-        SELECT 
-            GROUP_CONCAT(sample_id, ', ')
-            FROM Sample_List
-            WHERE "participant.study_participant_id" = sp.study_participant_id AND rn &lt;= 5
-    ), '') || 
-    CASE 
-        WHEN (SELECT COUNT(*) FROM Sample_List WHERE "participant.study_participant_id" = sp.study_participant_id) &gt; 5 
-        THEN ', ...' 
-        ELSE '' 
-    END AS "Sample Id",
-	f.file_type AS "File Type",
-    gi.library_strategy AS "Library Strategy",
-    '' AS "Supplementary Files"
-FROM Filtered_Files ff
-JOIN df_file f ON f.file_id = ff.file_id
-JOIN df_participant sp ON f."participant.study_participant_id" = sp.study_participant_id
-JOIN df_study s ON sp."study.phs_accession" = s.phs_accession
-JOIN df_genomic_info gi ON gi."file.file_id" = f.file_id
-JOIN df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-GROUP BY
-    f.file_name,
-    s.study_name,
-    s.phs_accession,
-    sp.participant_id,
-    f.file_type,
-    gi.library_strategy
-ORDER BY 
-    f.file_name ASC,
-    sp.participant_id ASC
-LIMIT 100;</t>
-  </si>
-  <si>
-    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_TSVData.xlsx</t>
-  </si>
-  <si>
-    <t>TC01_CDS_phs002599_SmpTumSta-NSD_SmpType-RNA_LibStr_TargetedCapture_WebData.xlsx</t>
-  </si>
-  <si>
-    <t>SELECT DISTINCT
-    smp.sample_id AS "Sample ID",
-    sp.participant_id AS "Participant ID", 
-    s.study_name AS "Study Name",
-    s.phs_accession AS Accession
-FROM 
-    df_participant sp
-JOIN 
-    df_study s ON sp."study.phs_accession" = s.phs_accession
-JOIN 
-    df_sample smp ON smp."participant.study_participant_id" = sp.study_participant_id
-JOIN 
-    df_file f1 ON f1."sample.sample_id" = smp.sample_id
-JOIN 
-    df_genomic_info gi ON gi."file.file_id" = f1.file_id
-JOIN 
-    df_diagnosis d ON d."participant.study_participant_id" = sp.study_participant_id
-JOIN 
-    df_program p ON p.program_acronym = s."program.program_acronym"
-WHERE 
-    s.phs_accession = 'phs002599' 
-    AND smp.sample_tumor_status = 'Not specified in data'
-    AND smp.sample_type = 'RNA'
-    AND gi.library_strategy = 'Targeted-Capture' 
-ORDER BY 
-    smp.sample_id ASC
-LIMIT 100;</t>
+    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+RETURN DISTINCT
+  s.study_acronym AS study_name,
+  s.phs_accession AS accession,
+  samp.sample_id AS sample_id,
+  COALESCE(samp.sample_name, samp.sample_id) AS sample_name,
+  COALESCE(samp.Organization_Name, "Not specified in data") AS organization_name
+ORDER BY samp.sample_id ASC
+LIMIT 100
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+WITH DISTINCT p, s
+OPTIONAL MATCH (samp_all:sample)-[:of_participant]-&gt;(p)
+WITH p, s, samp_all
+ORDER BY samp_all.sample_id ASC
+WITH p, s, [x IN collect(samp_all.sample_id) WHERE x IS NOT NULL] AS sample_ids
+WITH p, s, sample_ids,
+  CASE
+    WHEN size(sample_ids) &gt; 5
+    THEN reduce(acc = "", id IN sample_ids[0..5] | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END) + ", ..."
+    ELSE reduce(acc = "", id IN sample_ids | CASE WHEN acc = "" THEN id ELSE acc + ", " + id END)
+  END AS samples
+RETURN
+  p.participant_id AS participant_id,
+  s.study_name AS study_name,
+  s.phs_accession AS accession,
+  p.sex AS sex,
+  samples
+ORDER BY p.participant_id ASC
+LIMIT 100
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+  RETURN
+  count(DISTINCT s) AS Studies,
+  count(DISTINCT p) AS Participants,
+  count(DISTINCT samp) AS Samples,
+  count(DISTINCT f) AS Files
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATCH (samp:sample)-[:of_participant]-&gt;(p:participant)-[:of_study]-&gt;(s:study)
+MATCH (gi:genomic_info)-[:of_file]-&gt;(f:file)-[:of_participant]-&gt;(p)
+MATCH (f)-[:from_sample]-&gt;(samp)
+WHERE s.phs_accession = "phs002599"
+  AND samp.sample_tumor_status = "Not specified in data"
+  AND samp.sample_type = "RNA"
+RETURN DISTINCT
+  s.study_name AS study_name,
+  s.phs_accession AS accession,
+  f.file_name AS file_name,
+  f.file_id AS file_id,
+  f.file_type AS file_type,
+  COALESCE(samp.sample_id, "Not Applicable") AS sample_id
+ORDER BY f.file_name ASC
+LIMIT 100
+</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -282,12 +148,6 @@
     <font>
       <sz val="11"/>
       <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -326,7 +186,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -335,7 +195,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{7EA68BB1-159D-4F44-96A3-D0B7FBE8815D}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -646,78 +506,77 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C538400-E87C-4027-A918-A51DB80B3430}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="75.85546875" customWidth="1"/>
-    <col min="4" max="4" width="87.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="88.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="75.83203125" customWidth="1"/>
+    <col min="4" max="4" width="87.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="88.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:5" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="409.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C6" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>
 </file>
</xml_diff>